<commit_message>
Update university conversion rules and related files
</commit_message>
<xml_diff>
--- a/public/templates/student-record-template.xlsx
+++ b/public/templates/student-record-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\나\projects\susikok\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0215FF3-1306-43C3-9AC8-5432AB95D8BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD8F9E6-54A5-4B3F-8B91-32ADFE705BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="pE9hGmgvfe3J8+UxEz/hr5Px5upngUlAS33M+maH4CsISPSsP7HQaY+tzKO5rxqhLFM0qf6pPW5l3lIyK5eCSA==" workbookSaltValue="XzXO5VexvVUJlyEw7EESZw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="244">
   <si>
     <t>수시KOK 학생 성적 업로드 템플릿</t>
   </si>
@@ -1107,6 +1107,22 @@
   </si>
   <si>
     <t>학년학기, 교과, 이수구분을 순서대로 드롭다운하여 선택하면, 정확한 과목명을 확인한 후 선택 할 수 있습니다.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>재적수</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>A비율</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>B비율</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>C비율</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1197,8 +1213,8 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
-      <color theme="1"/>
+      <sz val="12"/>
+      <color theme="0"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
@@ -1330,32 +1346,32 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1660,58 +1676,66 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13407887-2213-4F01-9D3E-713EEBCE4164}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.19921875" style="9" customWidth="1"/>
-    <col min="2" max="2" width="12.5" style="9" customWidth="1"/>
-    <col min="3" max="3" width="14.796875" style="9" customWidth="1"/>
-    <col min="4" max="4" width="21.3984375" style="9" customWidth="1"/>
-    <col min="5" max="10" width="10.09765625" style="9" customWidth="1"/>
-    <col min="11" max="16384" width="8.796875" style="9"/>
+    <col min="1" max="1" width="16.19921875" style="13" customWidth="1"/>
+    <col min="2" max="2" width="12.5" style="13" customWidth="1"/>
+    <col min="3" max="3" width="14.796875" style="13" customWidth="1"/>
+    <col min="4" max="4" width="21.3984375" style="13" customWidth="1"/>
+    <col min="5" max="14" width="8.09765625" style="13" customWidth="1"/>
+    <col min="15" max="16384" width="8.796875" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:14" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-    </row>
-    <row r="2" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="13" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+    </row>
+    <row r="2" spans="1:14" ht="33" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-    </row>
-    <row r="3" spans="1:10" ht="6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="15"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-    </row>
-    <row r="4" spans="1:10" ht="21.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+    </row>
+    <row r="3" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+    </row>
+    <row r="4" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
         <v>1</v>
       </c>
@@ -1727,27 +1751,39 @@
       <c r="E4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="9" t="s">
         <v>238</v>
       </c>
       <c r="I4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="4" t="s">
-        <v>8</v>
+      <c r="K4" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="L4" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="M4" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="N4" s="16" t="s">
+        <v>243</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
     <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:N2"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="5">
@@ -1763,7 +1799,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5:D200" xr:uid="{F3A0F3F2-E11B-4184-938A-120C432E7843}">
       <formula1>INDIRECT($C5&amp;$B5)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I200" xr:uid="{17602E6B-9E4B-4D65-B178-E7998B90C21A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5:J200" xr:uid="{17602E6B-9E4B-4D65-B178-E7998B90C21A}">
       <formula1>성취도</formula1>
     </dataValidation>
   </dataValidations>
@@ -1828,7 +1864,7 @@
       <c r="I2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="12" t="s">
         <v>221</v>
       </c>
       <c r="K2" s="2" t="s">
@@ -1854,7 +1890,7 @@
       <c r="I3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="17"/>
+      <c r="J3" s="12"/>
       <c r="K3" s="2" t="s">
         <v>232</v>
       </c>
@@ -1878,7 +1914,7 @@
       <c r="I4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="17"/>
+      <c r="J4" s="12"/>
       <c r="K4" s="2" t="s">
         <v>233</v>
       </c>
@@ -1902,7 +1938,7 @@
       <c r="I5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="17"/>
+      <c r="J5" s="12"/>
       <c r="K5" s="2" t="s">
         <v>234</v>
       </c>
@@ -1926,7 +1962,7 @@
       <c r="I6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="J6" s="16" t="s">
+      <c r="J6" s="11" t="s">
         <v>222</v>
       </c>
       <c r="K6" s="2" t="s">
@@ -1952,7 +1988,7 @@
       <c r="I7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="16"/>
+      <c r="J7" s="11"/>
       <c r="K7" s="2" t="s">
         <v>236</v>
       </c>
@@ -1973,7 +2009,7 @@
       <c r="I8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="16"/>
+      <c r="J8" s="11"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
@@ -1991,7 +2027,7 @@
       <c r="I9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J9" s="16"/>
+      <c r="J9" s="11"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
@@ -2009,7 +2045,7 @@
       <c r="I10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="J10" s="17" t="s">
+      <c r="J10" s="12" t="s">
         <v>223</v>
       </c>
     </row>
@@ -2027,7 +2063,7 @@
       <c r="I11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J11" s="17"/>
+      <c r="J11" s="12"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
@@ -2043,7 +2079,7 @@
       <c r="I12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J12" s="17"/>
+      <c r="J12" s="12"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
@@ -2059,7 +2095,7 @@
       <c r="I13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="17"/>
+      <c r="J13" s="12"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
@@ -2075,7 +2111,7 @@
       <c r="I14" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="J14" s="16" t="s">
+      <c r="J14" s="11" t="s">
         <v>224</v>
       </c>
     </row>
@@ -2093,7 +2129,7 @@
       <c r="I15" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J15" s="16"/>
+      <c r="J15" s="11"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
@@ -2109,7 +2145,7 @@
       <c r="I16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J16" s="16"/>
+      <c r="J16" s="11"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
@@ -2125,7 +2161,7 @@
       <c r="I17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J17" s="16"/>
+      <c r="J17" s="11"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
@@ -2141,7 +2177,7 @@
       <c r="I18" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="J18" s="17" t="s">
+      <c r="J18" s="12" t="s">
         <v>225</v>
       </c>
     </row>
@@ -2159,7 +2195,7 @@
       <c r="I19" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J19" s="17"/>
+      <c r="J19" s="12"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A20" s="6" t="s">
@@ -2175,7 +2211,7 @@
       <c r="I20" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J20" s="17"/>
+      <c r="J20" s="12"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A21" s="6" t="s">
@@ -2191,7 +2227,7 @@
       <c r="I21" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J21" s="17"/>
+      <c r="J21" s="12"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A22" s="6" t="s">
@@ -2207,7 +2243,7 @@
       <c r="I22" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J22" s="16" t="s">
+      <c r="J22" s="11" t="s">
         <v>226</v>
       </c>
     </row>
@@ -2225,7 +2261,7 @@
       <c r="I23" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J23" s="16"/>
+      <c r="J23" s="11"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A24" s="6" t="s">
@@ -2241,7 +2277,7 @@
       <c r="I24" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J24" s="16"/>
+      <c r="J24" s="11"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A25" s="6" t="s">
@@ -2257,7 +2293,7 @@
       <c r="I25" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J25" s="17" t="s">
+      <c r="J25" s="12" t="s">
         <v>227</v>
       </c>
     </row>
@@ -2275,7 +2311,7 @@
       <c r="I26" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J26" s="17"/>
+      <c r="J26" s="12"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A27" s="6" t="s">
@@ -2291,7 +2327,7 @@
       <c r="I27" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J27" s="17"/>
+      <c r="J27" s="12"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A28" s="6" t="s">
@@ -2307,7 +2343,7 @@
       <c r="I28" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J28" s="16" t="s">
+      <c r="J28" s="11" t="s">
         <v>228</v>
       </c>
     </row>
@@ -2325,7 +2361,7 @@
       <c r="I29" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J29" s="16"/>
+      <c r="J29" s="11"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A30" s="6" t="s">
@@ -2341,7 +2377,7 @@
       <c r="I30" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J30" s="16"/>
+      <c r="J30" s="11"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A31" s="6" t="s">

</xml_diff>